<commit_message>
fixing the organization names and making lazyloads smaller
</commit_message>
<xml_diff>
--- a/data-raw/hrmis_data_dictionary.xlsx
+++ b/data-raw/hrmis_data_dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldbankgroup-my.sharepoint.com/personal/iedochie_worldbank_org/Documents/Documents/GitProjects/govhr/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="132" documentId="8_{19A0EA07-B73B-431C-B448-63D81EB501B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0AFC943B-A0D5-46AF-8DBE-BBF4D14F6899}"/>
+  <xr:revisionPtr revIDLastSave="138" documentId="8_{19A0EA07-B73B-431C-B448-63D81EB501B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01EC3345-096E-4139-9634-76F2CA4CAA5B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Establishment" sheetId="1" r:id="rId1"/>
@@ -22,15 +22,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="126">
   <si>
     <t>Description</t>
-  </si>
-  <si>
-    <t>Organization ID</t>
-  </si>
-  <si>
-    <t>org_id</t>
   </si>
   <si>
     <t>character</t>
@@ -477,7 +471,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -797,19 +791,19 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>124</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -817,189 +811,189 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D4" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
       <c r="E5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
         <v>123</v>
-      </c>
-      <c r="D6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D7" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D8" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D9" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D10" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D11" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D12" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1020,186 +1014,186 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" t="s">
         <v>116</v>
       </c>
-      <c r="B4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C4" t="s">
-        <v>118</v>
-      </c>
       <c r="E4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
       <c r="E5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D7" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D9" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D10" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D11" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1209,10 +1203,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.28515625" customWidth="1"/>
     <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -1220,410 +1214,427 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>87</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>94</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D5" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="D9" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B10" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C10" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D10" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>81</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>83</v>
       </c>
       <c r="D11" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D12" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D13" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D14" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D15" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B17" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C17" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="E17" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C18" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="E18" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C19" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D19" t="s">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>7</v>
+        <v>69</v>
       </c>
       <c r="B20" t="s">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="C20" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="D20" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="E20" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D21" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E21" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D22" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E22" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D23" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>11</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>12</v>
       </c>
       <c r="C24" t="s">
-        <v>79</v>
+        <v>13</v>
       </c>
       <c r="D24" t="s">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>127</v>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>72</v>
+      </c>
+      <c r="B25" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor rules and update dictionary
</commit_message>
<xml_diff>
--- a/data-raw/hrmis_data_dictionary.xlsx
+++ b/data-raw/hrmis_data_dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldbankgroup-my.sharepoint.com/personal/iedochie_worldbank_org/Documents/Documents/GitProjects/govhr/data-raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wb438023\github\govhr\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="138" documentId="8_{19A0EA07-B73B-431C-B448-63D81EB501B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01EC3345-096E-4139-9634-76F2CA4CAA5B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A27C7D4-1EBE-4EA5-9B4B-0CE0230828A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Establishment" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="124">
   <si>
     <t>Description</t>
   </si>
@@ -66,12 +66,6 @@
     <t>Code corresponding to the administrative division.</t>
   </si>
   <si>
-    <t>Worker ID</t>
-  </si>
-  <si>
-    <t>worker_id</t>
-  </si>
-  <si>
     <t>Date of the HRMIS record or data collection timestamp.</t>
   </si>
   <si>
@@ -138,24 +132,15 @@
     <t>Date of contract record entry.</t>
   </si>
   <si>
-    <t>Base Salary</t>
-  </si>
-  <si>
     <t>Basic pay before allowances and deductions.</t>
   </si>
   <si>
     <t>numeric</t>
   </si>
   <si>
-    <t>Gross Salary</t>
-  </si>
-  <si>
     <t>Total compensation before taxes and deductions.</t>
   </si>
   <si>
-    <t>Net Salary</t>
-  </si>
-  <si>
     <t>Take-home pay after taxes and deductions.</t>
   </si>
   <si>
@@ -240,9 +225,6 @@
     <t>Number of years in service or tenure within the organization.</t>
   </si>
   <si>
-    <t>Allowance</t>
-  </si>
-  <si>
     <t>allowance_lcu</t>
   </si>
   <si>
@@ -400,6 +382,18 @@
   </si>
   <si>
     <t>Contract</t>
+  </si>
+  <si>
+    <t>Base Salary (Local Currency Units)</t>
+  </si>
+  <si>
+    <t>Gross Salary (Local Currency Units)</t>
+  </si>
+  <si>
+    <t>Net Salary (Local Currency Units)</t>
+  </si>
+  <si>
+    <t>Allowance (Local Currency Units)</t>
   </si>
 </sst>
 </file>
@@ -489,10 +483,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -791,19 +781,19 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -811,53 +801,53 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" t="s">
         <v>92</v>
       </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
       <c r="D2" t="s">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="D4" t="s">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -868,64 +858,64 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" t="s">
         <v>89</v>
       </c>
-      <c r="B6" t="s">
-        <v>95</v>
-      </c>
       <c r="C6" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D6" t="s">
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" t="s">
         <v>90</v>
       </c>
-      <c r="B7" t="s">
-        <v>96</v>
-      </c>
       <c r="C7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D7" t="s">
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" t="s">
         <v>91</v>
       </c>
-      <c r="B8" t="s">
-        <v>97</v>
-      </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D8" t="s">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -936,13 +926,13 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D9" t="s">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -953,13 +943,13 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D10" t="s">
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -970,13 +960,13 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D11" t="s">
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -987,13 +977,13 @@
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="D12" t="s">
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -1014,67 +1004,67 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B2" t="s">
         <v>106</v>
       </c>
-      <c r="B2" t="s">
-        <v>112</v>
-      </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C3" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C4" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="E4" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1085,115 +1075,115 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D6" t="s">
         <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D8" t="s">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D9" t="s">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D10" t="s">
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D11" t="s">
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -1214,87 +1204,87 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" t="s">
-        <v>34</v>
-      </c>
       <c r="D2" t="s">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>100</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="D5" t="s">
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1305,339 +1295,340 @@
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
         <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E7" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E8" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>122</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="B10" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D10" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="B11" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="C11" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="D11" t="s">
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="D12" t="s">
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
         <v>1</v>
       </c>
       <c r="E13" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="D15" t="s">
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D16" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="B17" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D17" t="s">
         <v>4</v>
       </c>
       <c r="E17" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D18" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="E18" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D19" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E19" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C20" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="C21" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="D21" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E21" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C22" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D22" t="s">
         <v>1</v>
       </c>
       <c r="E22" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B23" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C23" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D23" t="s">
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="D24" t="s">
         <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>77</v>
+        <v>13</v>
       </c>
       <c r="D25" t="s">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="E25" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update dictionary Fixes #76
</commit_message>
<xml_diff>
--- a/data-raw/hrmis_data_dictionary.xlsx
+++ b/data-raw/hrmis_data_dictionary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wb438023\github\govhr\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB89B82-CAEB-4405-95BD-24886AFC7D2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C19B56-FF1C-4A59-81F1-FDCA8E376930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="130">
   <si>
     <t>Description</t>
   </si>
@@ -54,24 +54,15 @@
     <t>Administration 1 Name</t>
   </si>
   <si>
-    <t>adm1_name</t>
-  </si>
-  <si>
     <t>Administration 1 Code</t>
   </si>
   <si>
     <t>adm1_code</t>
   </si>
   <si>
-    <t>Date of the HRMIS record or data collection timestamp.</t>
-  </si>
-  <si>
     <t>Date of Birth</t>
   </si>
   <si>
-    <t>birth_day</t>
-  </si>
-  <si>
     <t>Gender</t>
   </si>
   <si>
@@ -81,9 +72,6 @@
     <t>educat7</t>
   </si>
   <si>
-    <t>Educational attainment in 7-level classification.</t>
-  </si>
-  <si>
     <t>Tribe</t>
   </si>
   <si>
@@ -99,24 +87,12 @@
     <t>Employment Status</t>
   </si>
   <si>
-    <t>status</t>
-  </si>
-  <si>
     <t>Contract ID</t>
   </si>
   <si>
     <t>contract_id</t>
   </si>
   <si>
-    <t>Unique identifier for each contract.</t>
-  </si>
-  <si>
-    <t>Worker associated with this contract.</t>
-  </si>
-  <si>
-    <t>Date of contract record entry.</t>
-  </si>
-  <si>
     <t>Basic pay before allowances and deductions.</t>
   </si>
   <si>
@@ -198,18 +174,6 @@
     <t>paygrade</t>
   </si>
   <si>
-    <t>Pay grade or salary scale classification.</t>
-  </si>
-  <si>
-    <t>Seniority</t>
-  </si>
-  <si>
-    <t>seniority</t>
-  </si>
-  <si>
-    <t>Number of years in service or tenure within the organization.</t>
-  </si>
-  <si>
     <t>allowance_lcu</t>
   </si>
   <si>
@@ -228,21 +192,12 @@
     <t>Contract Type Code</t>
   </si>
   <si>
-    <t>contract_type_code</t>
-  </si>
-  <si>
-    <t>Type of employment contract (PERM, FTERM, TEMP for active workers; INACTIVE, PENSIONERS for active workers)</t>
-  </si>
-  <si>
     <t>Contract Type (Native)</t>
   </si>
   <si>
     <t>contract_type_native</t>
   </si>
   <si>
-    <t>Type of employment conttract in native language</t>
-  </si>
-  <si>
     <t>Establishment ID</t>
   </si>
   <si>
@@ -258,15 +213,6 @@
     <t>Official Establishment name translated into English.</t>
   </si>
   <si>
-    <t>Type of Establishment</t>
-  </si>
-  <si>
-    <t>Parent Establishment ID</t>
-  </si>
-  <si>
-    <t>Child Establishment ID</t>
-  </si>
-  <si>
     <t>est_id</t>
   </si>
   <si>
@@ -276,72 +222,21 @@
     <t>est_name_english</t>
   </si>
   <si>
-    <t>est_type</t>
-  </si>
-  <si>
-    <t>est_parent</t>
-  </si>
-  <si>
-    <t>est_child</t>
-  </si>
-  <si>
-    <t>Unique identifier for the establishment</t>
-  </si>
-  <si>
-    <t>The latest date when the establishment had the specified name or attribute.</t>
-  </si>
-  <si>
-    <t>Identifier of the subordinate Establishment in hierachy</t>
-  </si>
-  <si>
-    <t>Identifier of the parent Establishment in hierarchy</t>
-  </si>
-  <si>
     <t>Official World Bank ISO 3-letter country code</t>
   </si>
   <si>
     <t>Official World Bank country name</t>
   </si>
   <si>
-    <t>First-level administrative division</t>
-  </si>
-  <si>
-    <t>First-level administrative division code</t>
-  </si>
-  <si>
     <t>Personnel ID</t>
   </si>
   <si>
-    <t>Personnel’s date of birth.</t>
-  </si>
-  <si>
-    <t>Sex of the Personnel.</t>
-  </si>
-  <si>
-    <t>Personnel’s ethnic or tribal affiliation.</t>
-  </si>
-  <si>
-    <t>Personnel’s race or broad ethnic classification.</t>
-  </si>
-  <si>
-    <t>Employment status of the Personnel (active, retired).</t>
-  </si>
-  <si>
     <t>personnel_id</t>
   </si>
   <si>
-    <t xml:space="preserve">Unique identifier assigned to each Personnel </t>
-  </si>
-  <si>
     <t>Foreign key linking to the establishment module</t>
   </si>
   <si>
-    <t>Educational Attainment (7-categories)</t>
-  </si>
-  <si>
-    <t>Type of establishment (either Ministry/Department/Agency)</t>
-  </si>
-  <si>
     <t>Module</t>
   </si>
   <si>
@@ -376,13 +271,154 @@
   </si>
   <si>
     <t>Variable Description</t>
+  </si>
+  <si>
+    <t>birth_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unique identifier assigned to each worker. </t>
+  </si>
+  <si>
+    <t>Unique identifier assigned to each contract.</t>
+  </si>
+  <si>
+    <t>Unique identifier assigned to each establishment.</t>
+  </si>
+  <si>
+    <t>Contract tenure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How much time a person has worked in a given contract. </t>
+  </si>
+  <si>
+    <t>Person tenure</t>
+  </si>
+  <si>
+    <t>How much time a person has worked in the public sector.</t>
+  </si>
+  <si>
+    <t>Person's race or broad ethnic classification.</t>
+  </si>
+  <si>
+    <t>Person's ethnic or tribal affiliation.</t>
+  </si>
+  <si>
+    <t>Gender of the person.</t>
+  </si>
+  <si>
+    <t>The date of birth of a person.</t>
+  </si>
+  <si>
+    <t>Date of the HRMIS record.</t>
+  </si>
+  <si>
+    <t>Educational Attainment</t>
+  </si>
+  <si>
+    <t>Educational attainment in 7-level classification, following the World Bank's GLD convention. Available here: https://worldbank.github.io/gld/Support/A%20-%20Guides%20and%20Documentation/GLD%20Manual%20Files/Education.html.</t>
+  </si>
+  <si>
+    <t>First-level administrative division code, if available</t>
+  </si>
+  <si>
+    <t>adm1</t>
+  </si>
+  <si>
+    <t>Administration 2 Name</t>
+  </si>
+  <si>
+    <t>Administration 2 Code</t>
+  </si>
+  <si>
+    <t>First-level administrative division. For example, a Ministry or Secretariat.</t>
+  </si>
+  <si>
+    <t>Second-level administrative division code, if available</t>
+  </si>
+  <si>
+    <t>adm2</t>
+  </si>
+  <si>
+    <t>adm2_code</t>
+  </si>
+  <si>
+    <t>adm3</t>
+  </si>
+  <si>
+    <t>adm3_code</t>
+  </si>
+  <si>
+    <t>Administration 3 Name</t>
+  </si>
+  <si>
+    <t>Administration 3 Code</t>
+  </si>
+  <si>
+    <t>Third-level administrative division code, if available</t>
+  </si>
+  <si>
+    <t>Third-level administrative division. For example, an Agency or Unit.</t>
+  </si>
+  <si>
+    <t>Second-level administrative division. For example, a Department or Division.</t>
+  </si>
+  <si>
+    <t>Geography 1 Name</t>
+  </si>
+  <si>
+    <t>geo1</t>
+  </si>
+  <si>
+    <t>First-level geographic division. For example, a state or region.</t>
+  </si>
+  <si>
+    <t>geo2</t>
+  </si>
+  <si>
+    <t>Geography 2 Name</t>
+  </si>
+  <si>
+    <t>Second-level geographic division. For example, a municipality or county.</t>
+  </si>
+  <si>
+    <t>Type of service</t>
+  </si>
+  <si>
+    <t>service_type</t>
+  </si>
+  <si>
+    <t>The type of service of a person: civilian or military.</t>
+  </si>
+  <si>
+    <t>personnel_tenure</t>
+  </si>
+  <si>
+    <t>contract_tenure</t>
+  </si>
+  <si>
+    <t>contract_type</t>
+  </si>
+  <si>
+    <t>Employment status of the person (active or retired).</t>
+  </si>
+  <si>
+    <t>employment_status</t>
+  </si>
+  <si>
+    <t>Type of employment contract. For example: indefinite (e.g., civil servant) or definite (e.g., intern).</t>
+  </si>
+  <si>
+    <t>Type of employment contract in native language.</t>
+  </si>
+  <si>
+    <t>Pay grade or salary scale classification of a contract.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -400,6 +436,12 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -761,7 +803,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
@@ -772,70 +814,70 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>117</v>
+        <v>82</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D2" t="s">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="B3" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="C4" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D4" t="s">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -846,142 +888,194 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D6" t="s">
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="D7" t="s">
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="D8" t="s">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>101</v>
       </c>
       <c r="B9" t="s">
-        <v>6</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D9" t="s">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>108</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>106</v>
       </c>
       <c r="C10" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="D10" t="s">
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>109</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="D11" t="s">
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>113</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>114</v>
       </c>
       <c r="C12" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="D12" t="s">
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>107</v>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>67</v>
+      </c>
+      <c r="D15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E15" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
@@ -992,53 +1086,53 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>117</v>
+        <v>82</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1049,125 +1143,160 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>83</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D6" t="s">
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>97</v>
       </c>
       <c r="D7" t="s">
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D8" t="s">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="D9" t="s">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" t="s">
         <v>24</v>
       </c>
-      <c r="B10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" t="s">
-        <v>100</v>
-      </c>
-      <c r="D10" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
-        <v>108</v>
+      <c r="E11" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" t="s">
+        <v>121</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
@@ -1178,325 +1307,342 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>85</v>
       </c>
       <c r="D2" t="s">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="B3" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="D4" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>109</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E6" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E7" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B9" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="D9" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>124</v>
       </c>
       <c r="C10" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
       <c r="D10" t="s">
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>128</v>
       </c>
       <c r="D11" t="s">
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="D12" t="s">
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
         <v>1</v>
       </c>
       <c r="E13" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D14" t="s">
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="D15" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
         <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="D17" t="s">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="E17" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E18" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="B19" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>129</v>
       </c>
       <c r="D19" t="s">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>109</v>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" t="s">
+        <v>123</v>
+      </c>
+      <c r="C20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D20" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enable native pipe in Positron R settings and update HRMIS data dictionary
</commit_message>
<xml_diff>
--- a/data-raw/hrmis_data_dictionary.xlsx
+++ b/data-raw/hrmis_data_dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wb438023\github\govhr\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldbankgroup-my.sharepoint.com/personal/iedochie_worldbank_org/Documents/Documents/GitProjects/govhr/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C19B56-FF1C-4A59-81F1-FDCA8E376930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="13_ncr:1_{F2C19B56-FF1C-4A59-81F1-FDCA8E376930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07D3FAD3-18DC-49FC-9CDD-FA81283FFB1A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Establishment" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="151">
   <si>
     <t>Description</t>
   </si>
@@ -129,9 +129,6 @@
     <t>occupation_isconame</t>
   </si>
   <si>
-    <t>Occupation mapped to ISCO classification.</t>
-  </si>
-  <si>
     <t>ISCO Code</t>
   </si>
   <si>
@@ -189,9 +186,6 @@
     <t>Allowances after salary has been paid</t>
   </si>
   <si>
-    <t>Contract Type Code</t>
-  </si>
-  <si>
     <t>Contract Type (Native)</t>
   </si>
   <si>
@@ -405,13 +399,82 @@
     <t>employment_status</t>
   </si>
   <si>
-    <t>Type of employment contract. For example: indefinite (e.g., civil servant) or definite (e.g., intern).</t>
-  </si>
-  <si>
     <t>Type of employment contract in native language.</t>
   </si>
   <si>
     <t>Pay grade or salary scale classification of a contract.</t>
+  </si>
+  <si>
+    <t>Values</t>
+  </si>
+  <si>
+    <t>native OR paste(est_id, personnel_id, sep = "-")</t>
+  </si>
+  <si>
+    <t>native</t>
+  </si>
+  <si>
+    <t>yyyy-mm-dd</t>
+  </si>
+  <si>
+    <t>Contract Type International</t>
+  </si>
+  <si>
+    <t>native translation to English</t>
+  </si>
+  <si>
+    <t>Occupation mapped to ISCO-08 classification.</t>
+  </si>
+  <si>
+    <t>ISCO classification names for Level 4</t>
+  </si>
+  <si>
+    <t>ISCO classification codes for Level 4</t>
+  </si>
+  <si>
+    <t>c("Permanent", "Fixed-Term", "Short-Term")</t>
+  </si>
+  <si>
+    <t>Type of employment contract following ILO standard ICSE-18 classifications. For example: permanent (e.g., civil servant) or short-term (e.g., intern).</t>
+  </si>
+  <si>
+    <t>c("active", "pensioner")</t>
+  </si>
+  <si>
+    <t>numeric in years</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>The age of the person</t>
+  </si>
+  <si>
+    <t>c("civilian", "military")</t>
+  </si>
+  <si>
+    <t>Sector</t>
+  </si>
+  <si>
+    <t>sector</t>
+  </si>
+  <si>
+    <t>World Bank convention ISO3-code</t>
+  </si>
+  <si>
+    <t>World Bank official name</t>
+  </si>
+  <si>
+    <t>c("No education", "Primary incomplete", "Primary complete", "Secondary incomplete", "Secondary complete", "Post-secondary but not university", "University (complete or incomplete)")</t>
+  </si>
+  <si>
+    <t>The COFOG sector classification an establishment belongs to at the adm1 level</t>
+  </si>
+  <si>
+    <t>c("General Public Services", "Defence", "Public order and safety", "Economic affairs", "Environmental protection", "Housing and community amenities", "Health", "Recreation, culture and religion", "Education", "Social protection")</t>
   </si>
 </sst>
 </file>
@@ -490,7 +553,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -499,6 +562,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -803,268 +869,335 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.28515625" customWidth="1"/>
+    <col min="3" max="3" width="28.140625" customWidth="1"/>
     <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>81</v>
-      </c>
       <c r="E1" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s">
         <v>58</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" t="s">
         <v>63</v>
       </c>
-      <c r="C2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C5" t="s">
+        <v>149</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>70</v>
+      </c>
+      <c r="F5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>96</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>107</v>
+      </c>
+      <c r="B12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B13" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F13" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
         <v>64</v>
       </c>
-      <c r="C3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="D15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
         <v>65</v>
       </c>
-      <c r="C4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C6" t="s">
-        <v>102</v>
-      </c>
-      <c r="D6" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s">
-        <v>98</v>
-      </c>
-      <c r="D7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>100</v>
-      </c>
-      <c r="B8" t="s">
-        <v>104</v>
-      </c>
-      <c r="C8" t="s">
-        <v>112</v>
-      </c>
-      <c r="D8" t="s">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>101</v>
-      </c>
-      <c r="B9" t="s">
-        <v>105</v>
-      </c>
-      <c r="C9" t="s">
-        <v>103</v>
-      </c>
-      <c r="D9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" t="s">
-        <v>111</v>
-      </c>
-      <c r="D10" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>109</v>
-      </c>
-      <c r="B11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C11" t="s">
-        <v>110</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1</v>
-      </c>
-      <c r="E11" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>113</v>
-      </c>
-      <c r="B12" t="s">
-        <v>114</v>
-      </c>
-      <c r="C12" t="s">
-        <v>115</v>
-      </c>
-      <c r="D12" t="s">
-        <v>1</v>
-      </c>
-      <c r="E12" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>117</v>
-      </c>
-      <c r="B13" t="s">
-        <v>116</v>
-      </c>
-      <c r="C13" t="s">
-        <v>118</v>
-      </c>
-      <c r="D13" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D14" t="s">
-        <v>1</v>
-      </c>
-      <c r="E14" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B15" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" t="s">
-        <v>67</v>
-      </c>
-      <c r="D15" t="s">
-        <v>1</v>
-      </c>
-      <c r="E15" t="s">
-        <v>72</v>
+      <c r="D16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -1075,67 +1208,78 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.140625" customWidth="1"/>
     <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" t="s">
         <v>82</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="F2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" t="s">
         <v>68</v>
       </c>
-      <c r="B2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
         <v>70</v>
       </c>
-      <c r="D3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1143,149 +1287,196 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D4" t="s">
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+      <c r="F4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+      <c r="F5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>140</v>
+      </c>
+      <c r="B6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="C6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D6" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" t="s">
         <v>15</v>
       </c>
-      <c r="C7" t="s">
-        <v>97</v>
-      </c>
-      <c r="D7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="C8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>16</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>17</v>
       </c>
-      <c r="C8" t="s">
-        <v>92</v>
-      </c>
-      <c r="D8" t="s">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="C9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>19</v>
       </c>
-      <c r="C9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="C10" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>71</v>
+      </c>
+      <c r="F10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>20</v>
       </c>
-      <c r="B10" t="s">
-        <v>126</v>
-      </c>
-      <c r="C10" t="s">
-        <v>125</v>
-      </c>
-      <c r="D10" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>89</v>
-      </c>
       <c r="B11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+      <c r="F11" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>119</v>
+        <v>87</v>
       </c>
       <c r="B12" t="s">
         <v>120</v>
       </c>
       <c r="C12" t="s">
-        <v>121</v>
+        <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>71</v>
+      </c>
+      <c r="F12" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
+        <v>71</v>
+      </c>
+      <c r="F13" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -1296,33 +1487,38 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.28515625" customWidth="1"/>
+    <col min="3" max="3" width="48.42578125" customWidth="1"/>
     <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="44" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1330,50 +1526,59 @@
         <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" t="s">
         <v>84</v>
       </c>
-      <c r="D3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" t="s">
-        <v>86</v>
-      </c>
       <c r="D4" t="s">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+      <c r="F4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1381,21 +1586,24 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C6" t="s">
         <v>23</v>
@@ -1404,15 +1612,18 @@
         <v>24</v>
       </c>
       <c r="E6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>76</v>
-      </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
@@ -1421,15 +1632,18 @@
         <v>24</v>
       </c>
       <c r="E7" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
         <v>26</v>
@@ -1438,61 +1652,73 @@
         <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D9" t="s">
         <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B10" t="s">
+        <v>122</v>
+      </c>
+      <c r="C10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" t="s">
         <v>55</v>
       </c>
-      <c r="B10" t="s">
-        <v>124</v>
-      </c>
-      <c r="C10" t="s">
-        <v>127</v>
-      </c>
-      <c r="D10" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" t="s">
-        <v>57</v>
-      </c>
       <c r="C11" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D11" t="s">
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -1506,10 +1732,13 @@
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -1523,10 +1752,13 @@
         <v>1</v>
       </c>
       <c r="E13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F13" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -1534,115 +1766,136 @@
         <v>34</v>
       </c>
       <c r="C14" t="s">
+        <v>133</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>35</v>
       </c>
-      <c r="D14" t="s">
-        <v>1</v>
-      </c>
-      <c r="E14" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
         <v>36</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>37</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E15" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>38</v>
       </c>
-      <c r="D15" t="s">
-        <v>1</v>
-      </c>
-      <c r="E15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
         <v>39</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>40</v>
-      </c>
-      <c r="C16" t="s">
-        <v>41</v>
       </c>
       <c r="D16" t="s">
         <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" t="s">
         <v>42</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>43</v>
-      </c>
-      <c r="C17" t="s">
-        <v>44</v>
       </c>
       <c r="D17" t="s">
         <v>4</v>
       </c>
       <c r="E17" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F17" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" t="s">
         <v>45</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>46</v>
-      </c>
-      <c r="C18" t="s">
-        <v>47</v>
       </c>
       <c r="D18" t="s">
         <v>24</v>
       </c>
       <c r="E18" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F18" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" t="s">
         <v>48</v>
       </c>
-      <c r="B19" t="s">
-        <v>49</v>
-      </c>
       <c r="C19" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D19" t="s">
         <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="F19" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B20" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C20" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D20" t="s">
         <v>24</v>
       </c>
       <c r="E20" t="s">
-        <v>74</v>
+        <v>72</v>
+      </c>
+      <c r="F20" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add TF-IDF/cosine `classify_text()` and integrate COFOG + allowance modules into Brazil HRMIS pipeline with updated dictionary/docs and data exports
</commit_message>
<xml_diff>
--- a/data-raw/hrmis_data_dictionary.xlsx
+++ b/data-raw/hrmis_data_dictionary.xlsx
@@ -8,24 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldbankgroup-my.sharepoint.com/personal/iedochie_worldbank_org/Documents/Documents/GitProjects/govhr/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="13_ncr:1_{F2C19B56-FF1C-4A59-81F1-FDCA8E376930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07D3FAD3-18DC-49FC-9CDD-FA81283FFB1A}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="13_ncr:1_{F2C19B56-FF1C-4A59-81F1-FDCA8E376930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EEE5789-D82F-4B3D-9BD4-208CC6EA01D6}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12960" yWindow="4320" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Establishment" sheetId="1" r:id="rId1"/>
     <sheet name="Personnel" sheetId="2" r:id="rId2"/>
     <sheet name="Contract" sheetId="3" r:id="rId3"/>
+    <sheet name="Supplementary" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="151">
-  <si>
-    <t>Description</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="162">
   <si>
     <t>character</t>
   </si>
@@ -228,9 +226,6 @@
     <t>personnel_id</t>
   </si>
   <si>
-    <t>Foreign key linking to the establishment module</t>
-  </si>
-  <si>
     <t>Module</t>
   </si>
   <si>
@@ -432,15 +427,9 @@
     <t>ISCO classification codes for Level 4</t>
   </si>
   <si>
-    <t>c("Permanent", "Fixed-Term", "Short-Term")</t>
-  </si>
-  <si>
     <t>Type of employment contract following ILO standard ICSE-18 classifications. For example: permanent (e.g., civil servant) or short-term (e.g., intern).</t>
   </si>
   <si>
-    <t>c("active", "pensioner")</t>
-  </si>
-  <si>
     <t>numeric in years</t>
   </si>
   <si>
@@ -468,13 +457,58 @@
     <t>World Bank official name</t>
   </si>
   <si>
-    <t>c("No education", "Primary incomplete", "Primary complete", "Secondary incomplete", "Secondary complete", "Post-secondary but not university", "University (complete or incomplete)")</t>
-  </si>
-  <si>
     <t>The COFOG sector classification an establishment belongs to at the adm1 level</t>
   </si>
   <si>
     <t>c("General Public Services", "Defence", "Public order and safety", "Economic affairs", "Environmental protection", "Housing and community amenities", "Health", "Recreation, culture and religion", "Education", "Social protection")</t>
+  </si>
+  <si>
+    <t>c("No education", "Primary incomplete", "Primary complete", "Secondary incomplete", "Secondary complete", "Post-secondary but not university", "University complete or incomplete")</t>
+  </si>
+  <si>
+    <t>allowance_type</t>
+  </si>
+  <si>
+    <t>Allowance Type</t>
+  </si>
+  <si>
+    <t>Allowance Value</t>
+  </si>
+  <si>
+    <t>Allowance value for the specific allowance type in local currency units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The allowance type </t>
+  </si>
+  <si>
+    <t>Allowance</t>
+  </si>
+  <si>
+    <t>first_employment_date</t>
+  </si>
+  <si>
+    <t>First Employment Date</t>
+  </si>
+  <si>
+    <t>Date personnel enter the public service for the first time</t>
+  </si>
+  <si>
+    <t>c("permanent", "fixed-term", "short-term", "pensioner", "inactive")</t>
+  </si>
+  <si>
+    <t>c("active", "inactive", "pensioner")</t>
+  </si>
+  <si>
+    <t>Seniority</t>
+  </si>
+  <si>
+    <t>seniority</t>
+  </si>
+  <si>
+    <t>The level within the paygrade of a specific contract</t>
+  </si>
+  <si>
+    <t>Identifier assigned to each person.</t>
   </si>
 </sst>
 </file>
@@ -553,7 +587,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -564,8 +598,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -874,7 +914,7 @@
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.140625" customWidth="1"/>
+    <col min="3" max="3" width="34.5703125" customWidth="1"/>
     <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="31.7109375" bestFit="1" customWidth="1"/>
@@ -882,322 +922,322 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>79</v>
-      </c>
       <c r="E1" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>127</v>
+        <v>67</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" t="s">
         <v>57</v>
       </c>
-      <c r="B3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" t="s">
-        <v>58</v>
-      </c>
       <c r="D3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" t="s">
         <v>59</v>
       </c>
-      <c r="B4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" t="s">
-        <v>60</v>
-      </c>
       <c r="D4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>140</v>
+      </c>
+      <c r="B5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" t="s">
         <v>144</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" t="s">
         <v>145</v>
-      </c>
-      <c r="C5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E5" t="s">
-        <v>70</v>
-      </c>
-      <c r="F5" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6" t="s">
         <v>3</v>
       </c>
-      <c r="C6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D6" t="s">
-        <v>4</v>
-      </c>
       <c r="E6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D7" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" t="s">
-        <v>11</v>
-      </c>
       <c r="C8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D8" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" t="s">
+        <v>101</v>
+      </c>
+      <c r="C10" t="s">
         <v>99</v>
       </c>
-      <c r="B10" t="s">
-        <v>103</v>
-      </c>
-      <c r="C10" t="s">
-        <v>101</v>
-      </c>
       <c r="D10" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F10" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D11" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F11" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D12" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" t="s">
+        <v>110</v>
+      </c>
+      <c r="C13" t="s">
         <v>111</v>
       </c>
-      <c r="B13" t="s">
-        <v>112</v>
-      </c>
-      <c r="C13" t="s">
-        <v>113</v>
-      </c>
       <c r="D13" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F13" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B14" t="s">
+        <v>112</v>
+      </c>
+      <c r="C14" t="s">
         <v>114</v>
       </c>
-      <c r="C14" t="s">
-        <v>116</v>
-      </c>
       <c r="D14" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F14" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
         <v>5</v>
       </c>
-      <c r="B15" t="s">
-        <v>6</v>
-      </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F15" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
         <v>7</v>
       </c>
-      <c r="B16" t="s">
-        <v>8</v>
-      </c>
       <c r="C16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F16" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -1209,274 +1249,269 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="37.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.140625" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="1" max="16384" width="37.85546875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="C4" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>71</v>
-      </c>
-      <c r="F2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>70</v>
-      </c>
-      <c r="F3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="F4" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F4" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C5" t="s">
-        <v>92</v>
-      </c>
-      <c r="D5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>140</v>
-      </c>
-      <c r="B6" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" t="s">
-        <v>142</v>
-      </c>
-      <c r="D6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" t="s">
-        <v>71</v>
-      </c>
-      <c r="F6" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" t="s">
-        <v>91</v>
-      </c>
-      <c r="D7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F7" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>94</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>95</v>
-      </c>
-      <c r="D8" t="s">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>90</v>
-      </c>
-      <c r="D9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>71</v>
-      </c>
-      <c r="F9" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s">
-        <v>89</v>
-      </c>
-      <c r="D10" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F10" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>124</v>
-      </c>
-      <c r="C11" t="s">
-        <v>123</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1</v>
-      </c>
-      <c r="E11" t="s">
-        <v>71</v>
-      </c>
-      <c r="F11" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B12" t="s">
-        <v>120</v>
-      </c>
-      <c r="C12" t="s">
-        <v>88</v>
-      </c>
-      <c r="D12" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" t="s">
-        <v>71</v>
-      </c>
-      <c r="F12" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>117</v>
-      </c>
-      <c r="B13" t="s">
-        <v>118</v>
-      </c>
-      <c r="C13" t="s">
-        <v>119</v>
-      </c>
-      <c r="D13" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
-        <v>71</v>
-      </c>
-      <c r="F13" t="s">
-        <v>143</v>
+      <c r="E13" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -1487,7 +1522,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" bestFit="1" customWidth="1"/>
@@ -1500,406 +1535,564 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>79</v>
-      </c>
       <c r="E1" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
-        <v>22</v>
-      </c>
       <c r="C2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" t="s">
         <v>66</v>
       </c>
-      <c r="B3" t="s">
-        <v>67</v>
-      </c>
       <c r="C3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="s">
         <v>70</v>
       </c>
       <c r="F4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" t="s">
-        <v>93</v>
-      </c>
-      <c r="D5" t="s">
-        <v>4</v>
-      </c>
       <c r="E5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
-        <v>24</v>
-      </c>
       <c r="E6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C10" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D10" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F10" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" t="s">
         <v>54</v>
       </c>
-      <c r="B11" t="s">
-        <v>55</v>
-      </c>
       <c r="C11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D11" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F11" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" t="s">
         <v>27</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>28</v>
       </c>
-      <c r="C12" t="s">
-        <v>29</v>
-      </c>
       <c r="D12" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" t="s">
         <v>30</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>31</v>
       </c>
-      <c r="C13" t="s">
-        <v>32</v>
-      </c>
       <c r="D13" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F13" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
         <v>33</v>
       </c>
-      <c r="B14" t="s">
-        <v>34</v>
-      </c>
       <c r="C14" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D14" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" t="s">
         <v>35</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>36</v>
       </c>
-      <c r="C15" t="s">
-        <v>37</v>
-      </c>
       <c r="D15" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" t="s">
         <v>38</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>39</v>
       </c>
-      <c r="C16" t="s">
-        <v>40</v>
-      </c>
       <c r="D16" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F16" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" t="s">
         <v>41</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>42</v>
       </c>
-      <c r="C17" t="s">
-        <v>43</v>
-      </c>
       <c r="D17" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F17" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" t="s">
         <v>44</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>45</v>
       </c>
-      <c r="C18" t="s">
-        <v>46</v>
-      </c>
       <c r="D18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E18" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F18" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" t="s">
         <v>47</v>
       </c>
-      <c r="B19" t="s">
-        <v>48</v>
-      </c>
       <c r="C19" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D19" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F19" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>158</v>
       </c>
       <c r="B20" t="s">
-        <v>121</v>
+        <v>159</v>
       </c>
       <c r="C20" t="s">
-        <v>86</v>
+        <v>160</v>
       </c>
       <c r="D20" t="s">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E20" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F20" t="s">
-        <v>129</v>
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" t="s">
+        <v>84</v>
+      </c>
+      <c r="D21" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" t="s">
+        <v>70</v>
+      </c>
+      <c r="F21" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B483C751-A96A-4DC0-BF08-40DBFED6663F}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="33.28515625" customWidth="1"/>
+    <col min="2" max="2" width="28.7109375" customWidth="1"/>
+    <col min="3" max="3" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>152</v>
+      </c>
+      <c r="F3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>152</v>
+      </c>
+      <c r="F4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B5" t="s">
+        <v>147</v>
+      </c>
+      <c r="C5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>152</v>
+      </c>
+      <c r="F5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>152</v>
+      </c>
+      <c r="F6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>